<commit_message>
Import exercise 2.1, disk sampling
</commit_message>
<xml_diff>
--- a/submitted_exercises.xlsx
+++ b/submitted_exercises.xlsx
@@ -4,7 +4,7 @@
   <fileVersion lastEdited="4" lowestEdited="4" rupBuild="3820"/>
   <workbookPr date1904="0"/>
   <bookViews>
-    <workbookView activeTab="0" windowWidth="9600" windowHeight="7600"/>
+    <workbookView activeTab="0" windowWidth="9600" windowHeight="7610"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -33157,21 +33157,25 @@
       </c>
       <c r="H12" s="11"/>
     </row>
-    <row r="13" spans="1:16384">
+    <row r="13" spans="1:16384" ht="18.75">
       <c r="A13" s="10">
         <v>1.3</v>
       </c>
-      <c r="B13" s="11"/>
+      <c r="B13" s="11">
+        <v>1</v>
+      </c>
       <c r="G13" s="10">
         <v>8.3000000000000007</v>
       </c>
       <c r="H13" s="11"/>
     </row>
-    <row r="14" spans="1:16384">
+    <row r="14" spans="1:16384" ht="18.75">
       <c r="A14" s="10">
         <v>1.3999999999999999</v>
       </c>
-      <c r="B14" s="11"/>
+      <c r="B14" s="11">
+        <v>1</v>
+      </c>
       <c r="D14" s="10">
         <v>7.0999999999999996</v>
       </c>
@@ -33187,11 +33191,13 @@
       </c>
       <c r="E15" s="11"/>
     </row>
-    <row r="16" spans="1:16384">
+    <row r="16" spans="1:16384" ht="18.75">
       <c r="A16" s="10">
         <v>2.1000000000000001</v>
       </c>
-      <c r="B16" s="11"/>
+      <c r="B16" s="11">
+        <v>1</v>
+      </c>
       <c r="G16" s="10">
         <v>9.0999999999999996</v>
       </c>
@@ -66106,7 +66112,7 @@
     <row r="34" spans="1:16384">
       <c r="B34" s="13">
         <f>SUM(B11:B31)</f>
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="C34" s="1"/>
       <c r="E34" s="13">
@@ -66135,7 +66141,7 @@
     <row r="38" spans="1:16384" ht="17.35">
       <c r="B38" s="14">
         <f>B34+E34+H34</f>
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="C38" s="16" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Import exercise 2.2, Box-Müller
</commit_message>
<xml_diff>
--- a/submitted_exercises.xlsx
+++ b/submitted_exercises.xlsx
@@ -33203,11 +33203,13 @@
       </c>
       <c r="H16" s="11"/>
     </row>
-    <row r="17" spans="1:16384">
+    <row r="17" spans="1:16384" ht="18.75">
       <c r="A17" s="10">
         <v>2.2000000000000002</v>
       </c>
-      <c r="B17" s="11"/>
+      <c r="B17" s="11">
+        <v>1</v>
+      </c>
       <c r="D17" s="10">
         <v>12.1</v>
       </c>
@@ -66112,7 +66114,7 @@
     <row r="34" spans="1:16384">
       <c r="B34" s="13">
         <f>SUM(B11:B31)</f>
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C34" s="1"/>
       <c r="E34" s="13">
@@ -66141,7 +66143,7 @@
     <row r="38" spans="1:16384" ht="17.35">
       <c r="B38" s="14">
         <f>B34+E34+H34</f>
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C38" s="16" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Update with partially done exercises
</commit_message>
<xml_diff>
--- a/submitted_exercises.xlsx
+++ b/submitted_exercises.xlsx
@@ -4,7 +4,7 @@
   <fileVersion lastEdited="4" lowestEdited="4" rupBuild="3820"/>
   <workbookPr date1904="0"/>
   <bookViews>
-    <workbookView activeTab="0" windowWidth="9600" windowHeight="7600"/>
+    <workbookView activeTab="0" windowWidth="19200" windowHeight="7600"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -33135,7 +33135,9 @@
       <c r="D11" s="10">
         <v>6.0999999999999996</v>
       </c>
-      <c r="E11" s="11"/>
+      <c r="E11" s="11">
+        <v>1</v>
+      </c>
       <c r="G11" s="10">
         <v>8.0999999999999996</v>
       </c>
@@ -33169,7 +33171,9 @@
       <c r="G13" s="10">
         <v>8.3000000000000007</v>
       </c>
-      <c r="H13" s="11"/>
+      <c r="H13" s="11">
+        <v>1</v>
+      </c>
     </row>
     <row r="14" spans="1:16384" ht="18.75">
       <c r="A14" s="10">
@@ -33181,17 +33185,23 @@
       <c r="D14" s="10">
         <v>7.0999999999999996</v>
       </c>
-      <c r="E14" s="11"/>
+      <c r="E14" s="11">
+        <v>1</v>
+      </c>
       <c r="G14" s="10">
         <v>8.4000000000000004</v>
       </c>
-      <c r="H14" s="11"/>
+      <c r="H14" s="11">
+        <v>1</v>
+      </c>
     </row>
-    <row r="15" spans="1:16384">
+    <row r="15" spans="1:16384" ht="18.75">
       <c r="D15" s="10">
         <v>7.2000000000000002</v>
       </c>
-      <c r="E15" s="11"/>
+      <c r="E15" s="11">
+        <v>1</v>
+      </c>
     </row>
     <row r="16" spans="1:16384" ht="18.75">
       <c r="A16" s="10">
@@ -33221,11 +33231,13 @@
       </c>
       <c r="H17" s="11"/>
     </row>
-    <row r="18" spans="1:16384">
+    <row r="18" spans="1:16384" ht="18.75">
       <c r="A18" s="10">
         <v>2.2999999999999998</v>
       </c>
-      <c r="B18" s="11"/>
+      <c r="B18" s="11">
+        <v>1</v>
+      </c>
       <c r="D18" s="10">
         <v>12.199999999999999</v>
       </c>
@@ -33241,11 +33253,13 @@
       </c>
       <c r="E19" s="11"/>
     </row>
-    <row r="20" spans="1:16384">
+    <row r="20" spans="1:16384" ht="18.75">
       <c r="A20" s="10">
         <v>3.1000000000000001</v>
       </c>
-      <c r="B20" s="11"/>
+      <c r="B20" s="11">
+        <v>1</v>
+      </c>
       <c r="D20" s="12" t="inlineStr">
         <is>
           <t>(opt) 12.4</t>
@@ -33257,21 +33271,25 @@
       </c>
       <c r="H20" s="11"/>
     </row>
-    <row r="21" spans="1:16384">
+    <row r="21" spans="1:16384" ht="18.75">
       <c r="A21" s="10">
         <v>3.2000000000000002</v>
       </c>
-      <c r="B21" s="11"/>
+      <c r="B21" s="11">
+        <v>1</v>
+      </c>
       <c r="G21" s="10">
         <v>10.199999999999999</v>
       </c>
       <c r="H21" s="11"/>
     </row>
-    <row r="22" spans="1:16384">
+    <row r="22" spans="1:16384" ht="18.75">
       <c r="A22" s="10">
         <v>3.2999999999999998</v>
       </c>
-      <c r="B22" s="11"/>
+      <c r="B22" s="11">
+        <v>1</v>
+      </c>
       <c r="D22" s="10">
         <v>13.1</v>
       </c>
@@ -66116,18 +66134,18 @@
     <row r="34" spans="1:16384">
       <c r="B34" s="13">
         <f>SUM(B11:B31)</f>
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="C34" s="1"/>
       <c r="E34" s="13">
         <f>SUM(E11:E31)</f>
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="F34" s="1"/>
       <c r="G34" s="1"/>
       <c r="H34" s="13">
         <f>SUM(H11:H31)</f>
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="37" spans="1:16384" ht="17.35">
@@ -66145,7 +66163,7 @@
     <row r="38" spans="1:16384" ht="17.35">
       <c r="B38" s="14">
         <f>B34+E34+H34</f>
-        <v>7</v>
+        <v>16</v>
       </c>
       <c r="C38" s="16" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Add 8.1 and 8.2 to tex file
</commit_message>
<xml_diff>
--- a/submitted_exercises.xlsx
+++ b/submitted_exercises.xlsx
@@ -33135,13 +33135,13 @@
       <c r="D11" s="10">
         <v>6.0999999999999996</v>
       </c>
-      <c r="E11" s="11">
-        <v>1</v>
-      </c>
+      <c r="E11" s="11"/>
       <c r="G11" s="10">
         <v>8.0999999999999996</v>
       </c>
-      <c r="H11" s="11"/>
+      <c r="H11" s="11">
+        <v>1</v>
+      </c>
     </row>
     <row r="12" spans="1:16384" ht="18.75">
       <c r="A12" s="10">
@@ -33171,9 +33171,7 @@
       <c r="G13" s="10">
         <v>8.3000000000000007</v>
       </c>
-      <c r="H13" s="11">
-        <v>1</v>
-      </c>
+      <c r="H13" s="11"/>
     </row>
     <row r="14" spans="1:16384" ht="18.75">
       <c r="A14" s="10">
@@ -33191,9 +33189,7 @@
       <c r="G14" s="10">
         <v>8.4000000000000004</v>
       </c>
-      <c r="H14" s="11">
-        <v>1</v>
-      </c>
+      <c r="H14" s="11"/>
     </row>
     <row r="15" spans="1:16384" ht="18.75">
       <c r="D15" s="10">
@@ -33281,9 +33277,7 @@
       <c r="G21" s="10">
         <v>10.199999999999999</v>
       </c>
-      <c r="H21" s="11">
-        <v>1</v>
-      </c>
+      <c r="H21" s="11"/>
     </row>
     <row r="22" spans="1:16384" ht="18.75">
       <c r="A22" s="10">
@@ -33307,41 +33301,49 @@
       </c>
       <c r="E23" s="11"/>
     </row>
-    <row r="24" spans="1:16384">
+    <row r="24" spans="1:16384" ht="18.75">
       <c r="A24" s="10">
         <v>4.0999999999999996</v>
       </c>
-      <c r="B24" s="11"/>
+      <c r="B24" s="11">
+        <v>1</v>
+      </c>
       <c r="G24" s="10">
         <v>11.1</v>
       </c>
       <c r="H24" s="11"/>
     </row>
-    <row r="25" spans="1:16384">
+    <row r="25" spans="1:16384" ht="18.75">
       <c r="A25" s="10">
         <v>4.2000000000000002</v>
       </c>
-      <c r="B25" s="11"/>
+      <c r="B25" s="11">
+        <v>1</v>
+      </c>
       <c r="G25" s="10">
         <v>11.199999999999999</v>
       </c>
       <c r="H25" s="11"/>
     </row>
-    <row r="26" spans="1:16384">
+    <row r="26" spans="1:16384" ht="18.75">
       <c r="A26" s="10">
         <v>4.2999999999999998</v>
       </c>
-      <c r="B26" s="11"/>
+      <c r="B26" s="11">
+        <v>1</v>
+      </c>
       <c r="G26" s="10">
         <v>11.300000000000001</v>
       </c>
       <c r="H26" s="11"/>
     </row>
-    <row r="27" spans="1:16384">
+    <row r="27" spans="1:16384" ht="18.75">
       <c r="A27" s="10">
         <v>4.4000000000000004</v>
       </c>
-      <c r="B27" s="11"/>
+      <c r="B27" s="11">
+        <v>1</v>
+      </c>
       <c r="I27" s="1"/>
       <c r="J27" s="1"/>
       <c r="K27" s="1"/>
@@ -49719,11 +49721,13 @@
       <c r="XFC27" s="1"/>
       <c r="XFD27" s="1"/>
     </row>
-    <row r="28" spans="1:16384">
+    <row r="28" spans="1:16384" ht="18.75">
       <c r="A28" s="10">
         <v>4.5</v>
       </c>
-      <c r="B28" s="11"/>
+      <c r="B28" s="11">
+        <v>1</v>
+      </c>
       <c r="I28" s="1"/>
       <c r="J28" s="1"/>
       <c r="K28" s="1"/>
@@ -66136,18 +66140,18 @@
     <row r="34" spans="1:16384">
       <c r="B34" s="13">
         <f>SUM(B11:B31)</f>
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="C34" s="1"/>
       <c r="E34" s="13">
         <f>SUM(E11:E31)</f>
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F34" s="1"/>
       <c r="G34" s="1"/>
       <c r="H34" s="13">
         <f>SUM(H11:H31)</f>
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="37" spans="1:16384" ht="17.35">
@@ -66165,7 +66169,7 @@
     <row r="38" spans="1:16384" ht="17.35">
       <c r="B38" s="14">
         <f>B34+E34+H34</f>
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="C38" s="16" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Finish writing about 6.1
</commit_message>
<xml_diff>
--- a/submitted_exercises.xlsx
+++ b/submitted_exercises.xlsx
@@ -33135,7 +33135,9 @@
       <c r="D11" s="10">
         <v>6.0999999999999996</v>
       </c>
-      <c r="E11" s="11"/>
+      <c r="E11" s="11">
+        <v>1</v>
+      </c>
       <c r="G11" s="10">
         <v>8.0999999999999996</v>
       </c>
@@ -66145,7 +66147,7 @@
       <c r="C34" s="1"/>
       <c r="E34" s="13">
         <f>SUM(E11:E31)</f>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F34" s="1"/>
       <c r="G34" s="1"/>
@@ -66169,7 +66171,7 @@
     <row r="38" spans="1:16384" ht="17.35">
       <c r="B38" s="14">
         <f>B34+E34+H34</f>
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C38" s="16" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Finish writing exercise 8.4
</commit_message>
<xml_diff>
--- a/submitted_exercises.xlsx
+++ b/submitted_exercises.xlsx
@@ -33193,7 +33193,9 @@
       <c r="G14" s="10">
         <v>8.4000000000000004</v>
       </c>
-      <c r="H14" s="11"/>
+      <c r="H14" s="11">
+        <v>1</v>
+      </c>
     </row>
     <row r="15" spans="1:16384" ht="18.75">
       <c r="D15" s="10">
@@ -66155,7 +66157,7 @@
       <c r="G34" s="1"/>
       <c r="H34" s="13">
         <f>SUM(H11:H31)</f>
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="37" spans="1:16384" ht="17.35">
@@ -66173,7 +66175,7 @@
     <row r="38" spans="1:16384" ht="17.35">
       <c r="B38" s="14">
         <f>B34+E34+H34</f>
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="C38" s="16" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Finish writing exercises 9.2 and 9.3
</commit_message>
<xml_diff>
--- a/submitted_exercises.xlsx
+++ b/submitted_exercises.xlsx
@@ -33233,7 +33233,9 @@
       <c r="G17" s="10">
         <v>9.1999999999999993</v>
       </c>
-      <c r="H17" s="11"/>
+      <c r="H17" s="11">
+        <v>1</v>
+      </c>
     </row>
     <row r="18" spans="1:16384" ht="18.75">
       <c r="A18" s="10">
@@ -33249,7 +33251,9 @@
       <c r="G18" s="10">
         <v>9.3000000000000007</v>
       </c>
-      <c r="H18" s="11"/>
+      <c r="H18" s="11">
+        <v>1</v>
+      </c>
     </row>
     <row r="19" spans="1:16384">
       <c r="D19" s="10">
@@ -66159,7 +66163,7 @@
       <c r="G34" s="1"/>
       <c r="H34" s="13">
         <f>SUM(H11:H31)</f>
-        <v>5</v>
+        <v>7</v>
       </c>
     </row>
     <row r="37" spans="1:16384" ht="17.35">
@@ -66177,7 +66181,7 @@
     <row r="38" spans="1:16384" ht="17.35">
       <c r="B38" s="14">
         <f>B34+E34+H34</f>
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="C38" s="16" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Finish writing exercise 10.3
</commit_message>
<xml_diff>
--- a/submitted_exercises.xlsx
+++ b/submitted_exercises.xlsx
@@ -33309,7 +33309,9 @@
       <c r="G22" s="10">
         <v>10.300000000000001</v>
       </c>
-      <c r="H22" s="11"/>
+      <c r="H22" s="11">
+        <v>1</v>
+      </c>
     </row>
     <row r="23" spans="1:16384">
       <c r="D23" s="10">
@@ -66167,7 +66169,7 @@
       <c r="G34" s="1"/>
       <c r="H34" s="13">
         <f>SUM(H11:H31)</f>
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="37" spans="1:16384" ht="17.35">
@@ -66185,7 +66187,7 @@
     <row r="38" spans="1:16384" ht="17.35">
       <c r="B38" s="14">
         <f>B34+E34+H34</f>
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="C38" s="16" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Finish writing exercise 12.2
</commit_message>
<xml_diff>
--- a/submitted_exercises.xlsx
+++ b/submitted_exercises.xlsx
@@ -239,7 +239,7 @@
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
   <dimension ref="A1:XFD38"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="67.5" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" style="1" width="10.55" customWidth="1"/>
     <col min="2" max="2" style="2" width="10.55" customWidth="1"/>
@@ -33249,7 +33249,9 @@
       <c r="D18" s="10">
         <v>12.199999999999999</v>
       </c>
-      <c r="E18" s="11"/>
+      <c r="E18" s="11">
+        <v>1</v>
+      </c>
       <c r="G18" s="10">
         <v>9.3000000000000007</v>
       </c>
@@ -66167,7 +66169,7 @@
       <c r="C34" s="1"/>
       <c r="E34" s="13">
         <f>SUM(E11:E31)</f>
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F34" s="1"/>
       <c r="G34" s="1"/>
@@ -66191,7 +66193,7 @@
     <row r="38" spans="1:16384" ht="17.35">
       <c r="B38" s="14">
         <f>B34+E34+H34</f>
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="C38" s="16" t="inlineStr">
         <is>

</xml_diff>